<commit_message>
prg Fri Jun  5 11:38:37 AM CEST 2026
</commit_message>
<xml_diff>
--- a/public/routers/A0_Sistema_FV/A61_Conectado_a_red/FV04_Probando.xlsx
+++ b/public/routers/A0_Sistema_FV/A61_Conectado_a_red/FV04_Probando.xlsx
@@ -8,7 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="PDF" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="COSTES_DE_INSTALACION" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Diseño_FV" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CONSUMO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="COSTES_DE_INSTALACION" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="COSTES_DE_OPERACION" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="INGRESOS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="FINANCIEROS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -591,7 +596,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>pperez@instalaciones.com</t>
+          <t>pperezinstalaciones.com</t>
         </is>
       </c>
     </row>
@@ -656,7 +661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:AG3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -672,33 +677,842 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Variable</t>
+          <t>name</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Fijo (€)</t>
+          <t>tipoEstructura</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>valor</t>
+          <t>id</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Ud</t>
+          <t>lat</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>MO (%)</t>
+          <t>lng</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>rotation</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>width</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>height</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>tilt</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>slope</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>orientation</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>modelo</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>potenciaW</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>cols</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>inverterModel</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>inverterPower</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>mpptCount</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>vOc</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>vMp</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>iSc</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>iMp</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>coefVoc</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>vMax</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>vMinMppt</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>vMaxMppt</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>iMaxInverter</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>iScMaxInverter</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>paneles</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>sombras</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>geojson</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>FV</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Paneles</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>G1c</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>coplanar</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1779618894878</v>
+      </c>
+      <c r="F2" t="n">
+        <v>36.66629732748714</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-4.460736215114594</v>
+      </c>
+      <c r="H2" t="n">
+        <v>35.77607771789466</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1.134</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2.063</v>
+      </c>
+      <c r="K2" t="n">
+        <v>30</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>vertical</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>JAM60D42-LB</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>540</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Deye SUN-5K-SG05 LP1-EU-AM2-P</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U2" t="n">
+        <v>44.33</v>
+      </c>
+      <c r="V2" t="n">
+        <v>37.25</v>
+      </c>
+      <c r="W2" t="n">
+        <v>15.36</v>
+      </c>
+      <c r="X2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>500</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>150</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>425</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>18</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>27</v>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>['0,0','0,1','0,2','0,3','0,4','-1,5','-1,6','-1,4','-2,4','-2,5']</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>[1,1,40,45,50,55,1,1,1,1,1,1,1,1,1,1]</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>{'type':'FeatureCollection','features':[{'type':'Feature','properties':{'area':'G1c','block':'0,0'},'geometry':{'type':'Polygon','coordinates':[[[-4.460747215547954,36.66629379471248],[-4.460736912056057,36.666287839260065],[-4.460725214681235,36.666300860261806],[-4.460735518173132,36.66630681571422],[-4.460747215547954,36.66629379471248]]]}},{'type':'Feature','properties':{'area':'G1c','block':'0,1'},'geometry':{'type':'Polygon','coordinates':[[[-4.460736912056057,36.666287839260065],[-4.460726608564159,36.66628188380764],[-4.460714911189337,36.666294904809384],[-4.460725214681235,36.666300860261806],[-4.460736912056057,36.666287839260065]]]}},{'type':'Feature','properties':{'area':'G1c','block':'0,2'},'geometry':{'type':'Polygon','coordinates':[[[-4.460726608564159,36.66628188380764],[-4.460716305072261,36.666275928355226],[-4.460704607697439,36.66628894935697],[-4.460714911189337,36.666294904809384],[-4.460726608564159,36.66628188380764]]]}},{'type':'Feature','properties':{'area':'G1c','block':'0,3'},'geometry':{'type':'Polygon','coordinates':[[[-4.460716305072261,36.666275928355226],[-4.4607060015803635,36.6662699729028],[-4.460694304205541,36.666282993904545],[-4.460704607697439,36.66628894935697],[-4.460716305072261,36.666275928355226]]]}},{'type':'Feature','properties':{'area':'G1c','block':'0,4'},'geometry':{'type':'Polygon','coordinates':[[[-4.4607060015803635,36.6662699729028],[-4.4606956980884656,36.66626401745039],[-4.460684000713643,36.66627703845213],[-4.460694304205541,36.666282993904545],[-4.4607060015803635,36.6662699729028]]]}},{'type':'Feature','properties':{'area':'G1c','block':'-1,5'},'geometry':{'type':'Polygon','coordinates':[[[-4.460684000713643,36.66627703845213],[-4.460673697221745,36.66627108299971],[-4.460661999846923,36.66628410400145],[-4.4606723033388205,36.66629005945387],[-4.460684000713643,36.66627703845213]]]}},{'type':'Feature','properties':{'area':'G1c','block':'-1,6'},'geometry':{'type':'Polygon','coordinates':[[[-4.460673697221745,36.66627108299971],[-4.460663393729847,36.66626512754729],[-4.460651696355025,36.66627814854903],[-4.460661999846923,36.66628410400145],[-4.460673697221745,36.66627108299971]]]}},{'type':'Feature','properties':{'area':'G1c','block':'-1,4'},'geometry':{'type':'Polygon','coordinates':[[[-4.460694304205541,36.666282993904545],[-4.460684000713643,36.66627703845213],[-4.4606723033388205,36.66629005945387],[-4.460682606830718,36.66629601490629],[-4.460694304205541,36.666282993904545]]]}},{'type':'Feature','properties':{'area':'G1c','block':'-2,4'},'geometry':{'type':'Polygon','coordinates':[[[-4.460682606830718,36.66629601490629],[-4.4606723033388205,36.66629005945387],[-4.460660605963998,36.66630308045561],[-4.460670909455896,36.66630903590803],[-4.460682606830718,36.66629601490629]]]}},{'type':'Feature','properties':{'area':'G1c','block':'-2,5'},'geometry':{'type':'Polygon','coordinates':[[[-4.4606723033388205,36.66629005945387],[-4.460661999846923,36.66628410400145],[-4.4606503024721,36.66629712500319],[-4.460660605963998,36.66630308045561],[-4.4606723033388205,36.66629005945387]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,0'},'geometry':{'type':'Polygon','coordinates':[[[-4.460735816163178,36.666318536640915],[-4.460725512667968,36.6663125811885],[-4.460713815289385,36.66632560219024],[-4.4607241187845945,36.66633155764266],[-4.460735816163178,36.666318536640915]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,1'},'geometry':{'type':'Polygon','coordinates':[[[-4.460725512667968,36.6663125811885],[-4.460715209172757,36.66630662573608],[-4.460703511794175,36.66631964673782],[-4.460713815289385,36.66632560219024],[-4.460725512667968,36.6663125811885]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,2'},'geometry':{'type':'Polygon','coordinates':[[[-4.460715209172757,36.66630662573608],[-4.460704905677547,36.66630067028366],[-4.460693208298964,36.6663136912854],[-4.460703511794175,36.66631964673782],[-4.460715209172757,36.66630662573608]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,3'},'geometry':{'type':'Polygon','coordinates':[[[-4.460704905677547,36.66630067028366],[-4.460694602182337,36.66629471483124],[-4.460682904803754,36.66630773583298],[-4.460693208298964,36.6663136912854],[-4.460704905677547,36.66630067028366]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,4'},'geometry':{'type':'Polygon','coordinates':[[[-4.460694602182337,36.66629471483124],[-4.460684298687127,36.66628875937882],[-4.460672601308544,36.666301780380564],[-4.460682904803754,36.66630773583298],[-4.460694602182337,36.66629471483124]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,3'},'geometry':{'type':'Polygon','coordinates':[[[-4.460693208298964,36.6663136912854],[-4.460682904803754,36.66630773583298],[-4.460671207425171,36.66632075683472],[-4.460681510920381,36.666326712287145],[-4.460693208298964,36.6663136912854]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,2'},'geometry':{'type':'Polygon','coordinates':[[[-4.460703511794175,36.66631964673782],[-4.460693208298964,36.6663136912854],[-4.460681510920381,36.666326712287145],[-4.460691814415592,36.66633266773956],[-4.460703511794175,36.66631964673782]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,1'},'geometry':{'type':'Polygon','coordinates':[[[-4.460713815289385,36.66632560219024],[-4.460703511794175,36.66631964673782],[-4.460691814415592,36.66633266773956],[-4.4607021179108015,36.66633862319198],[-4.460713815289385,36.66632560219024]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,0'},'geometry':{'type':'Polygon','coordinates':[[[-4.4607241187845945,36.66633155764266],[-4.460713815289385,36.66632560219024],[-4.4607021179108015,36.66633862319198],[-4.460712421406011,36.6663445786444],[-4.4607241187845945,36.66633155764266]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,-1'},'geometry':{'type':'Polygon','coordinates':[[[-4.460734422279805,36.66633751309508],[-4.4607241187845945,36.66633155764266],[-4.460712421406011,36.6663445786444],[-4.460722724901222,36.66635053409682],[-4.460734422279805,36.66633751309508]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,5'},'geometry':{'type':'Polygon','coordinates':[[[-4.460684298687127,36.66628875937882],[-4.460673995191916,36.6662828039264],[-4.460662297813333,36.66629582492814],[-4.460672601308544,36.666301780380564],[-4.460684298687127,36.66628875937882]]]}}]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FV</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Paneles</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>coplanar</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1779618775455</v>
+      </c>
+      <c r="F3" t="n">
+        <v>36.66632206941558</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-4.460724815726281</v>
+      </c>
+      <c r="H3" t="n">
+        <v>35.77607771789466</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1.134</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2.063</v>
+      </c>
+      <c r="K3" t="n">
+        <v>30</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>vertical</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>JAM60D42-LB</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>540</v>
+      </c>
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Deye SUN-5K-SG05 LP1-EU-AM2-P</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="T3" t="n">
+        <v>2</v>
+      </c>
+      <c r="U3" t="n">
+        <v>44.33</v>
+      </c>
+      <c r="V3" t="n">
+        <v>37.25</v>
+      </c>
+      <c r="W3" t="n">
+        <v>15.36</v>
+      </c>
+      <c r="X3" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>500</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>150</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>425</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>18</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>27</v>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>['0,0','0,1','0,2','0,3','0,4','-1,3','-1,2','-1,1','-1,0','-1,-1','0,5']</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>[1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1]</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>{'type':'FeatureCollection','features':[{'type':'Feature','properties':{'area':'G1c','block':'0,0'},'geometry':{'type':'Polygon','coordinates':[[[-4.460747215547954,36.66629379471248],[-4.460736912056057,36.666287839260065],[-4.460725214681235,36.666300860261806],[-4.460735518173132,36.66630681571422],[-4.460747215547954,36.66629379471248]]]}},{'type':'Feature','properties':{'area':'G1c','block':'0,1'},'geometry':{'type':'Polygon','coordinates':[[[-4.460736912056057,36.666287839260065],[-4.460726608564159,36.66628188380764],[-4.460714911189337,36.666294904809384],[-4.460725214681235,36.666300860261806],[-4.460736912056057,36.666287839260065]]]}},{'type':'Feature','properties':{'area':'G1c','block':'0,2'},'geometry':{'type':'Polygon','coordinates':[[[-4.460726608564159,36.66628188380764],[-4.460716305072261,36.666275928355226],[-4.460704607697439,36.66628894935697],[-4.460714911189337,36.666294904809384],[-4.460726608564159,36.66628188380764]]]}},{'type':'Feature','properties':{'area':'G1c','block':'0,3'},'geometry':{'type':'Polygon','coordinates':[[[-4.460716305072261,36.666275928355226],[-4.4607060015803635,36.6662699729028],[-4.460694304205541,36.666282993904545],[-4.460704607697439,36.66628894935697],[-4.460716305072261,36.666275928355226]]]}},{'type':'Feature','properties':{'area':'G1c','block':'0,4'},'geometry':{'type':'Polygon','coordinates':[[[-4.4607060015803635,36.6662699729028],[-4.4606956980884656,36.66626401745039],[-4.460684000713643,36.66627703845213],[-4.460694304205541,36.666282993904545],[-4.4607060015803635,36.6662699729028]]]}},{'type':'Feature','properties':{'area':'G1c','block':'-1,5'},'geometry':{'type':'Polygon','coordinates':[[[-4.460684000713643,36.66627703845213],[-4.460673697221745,36.66627108299971],[-4.460661999846923,36.66628410400145],[-4.4606723033388205,36.66629005945387],[-4.460684000713643,36.66627703845213]]]}},{'type':'Feature','properties':{'area':'G1c','block':'-1,6'},'geometry':{'type':'Polygon','coordinates':[[[-4.460673697221745,36.66627108299971],[-4.460663393729847,36.66626512754729],[-4.460651696355025,36.66627814854903],[-4.460661999846923,36.66628410400145],[-4.460673697221745,36.66627108299971]]]}},{'type':'Feature','properties':{'area':'G1c','block':'-1,4'},'geometry':{'type':'Polygon','coordinates':[[[-4.460694304205541,36.666282993904545],[-4.460684000713643,36.66627703845213],[-4.4606723033388205,36.66629005945387],[-4.460682606830718,36.66629601490629],[-4.460694304205541,36.666282993904545]]]}},{'type':'Feature','properties':{'area':'G1c','block':'-2,4'},'geometry':{'type':'Polygon','coordinates':[[[-4.460682606830718,36.66629601490629],[-4.4606723033388205,36.66629005945387],[-4.460660605963998,36.66630308045561],[-4.460670909455896,36.66630903590803],[-4.460682606830718,36.66629601490629]]]}},{'type':'Feature','properties':{'area':'G1c','block':'-2,5'},'geometry':{'type':'Polygon','coordinates':[[[-4.4606723033388205,36.66629005945387],[-4.460661999846923,36.66628410400145],[-4.4606503024721,36.66629712500319],[-4.460660605963998,36.66630308045561],[-4.4606723033388205,36.66629005945387]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,0'},'geometry':{'type':'Polygon','coordinates':[[[-4.460735816163178,36.666318536640915],[-4.460725512667968,36.6663125811885],[-4.460713815289385,36.66632560219024],[-4.4607241187845945,36.66633155764266],[-4.460735816163178,36.666318536640915]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,1'},'geometry':{'type':'Polygon','coordinates':[[[-4.460725512667968,36.6663125811885],[-4.460715209172757,36.66630662573608],[-4.460703511794175,36.66631964673782],[-4.460713815289385,36.66632560219024],[-4.460725512667968,36.6663125811885]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,2'},'geometry':{'type':'Polygon','coordinates':[[[-4.460715209172757,36.66630662573608],[-4.460704905677547,36.66630067028366],[-4.460693208298964,36.6663136912854],[-4.460703511794175,36.66631964673782],[-4.460715209172757,36.66630662573608]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,3'},'geometry':{'type':'Polygon','coordinates':[[[-4.460704905677547,36.66630067028366],[-4.460694602182337,36.66629471483124],[-4.460682904803754,36.66630773583298],[-4.460693208298964,36.6663136912854],[-4.460704905677547,36.66630067028366]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,4'},'geometry':{'type':'Polygon','coordinates':[[[-4.460694602182337,36.66629471483124],[-4.460684298687127,36.66628875937882],[-4.460672601308544,36.666301780380564],[-4.460682904803754,36.66630773583298],[-4.460694602182337,36.66629471483124]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,3'},'geometry':{'type':'Polygon','coordinates':[[[-4.460693208298964,36.6663136912854],[-4.460682904803754,36.66630773583298],[-4.460671207425171,36.66632075683472],[-4.460681510920381,36.666326712287145],[-4.460693208298964,36.6663136912854]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,2'},'geometry':{'type':'Polygon','coordinates':[[[-4.460703511794175,36.66631964673782],[-4.460693208298964,36.6663136912854],[-4.460681510920381,36.666326712287145],[-4.460691814415592,36.66633266773956],[-4.460703511794175,36.66631964673782]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,1'},'geometry':{'type':'Polygon','coordinates':[[[-4.460713815289385,36.66632560219024],[-4.460703511794175,36.66631964673782],[-4.460691814415592,36.66633266773956],[-4.4607021179108015,36.66633862319198],[-4.460713815289385,36.66632560219024]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,0'},'geometry':{'type':'Polygon','coordinates':[[[-4.4607241187845945,36.66633155764266],[-4.460713815289385,36.66632560219024],[-4.4607021179108015,36.66633862319198],[-4.460712421406011,36.6663445786444],[-4.4607241187845945,36.66633155764266]]]}},{'type':'Feature','properties':{'area':'G1','block':'-1,-1'},'geometry':{'type':'Polygon','coordinates':[[[-4.460734422279805,36.66633751309508],[-4.4607241187845945,36.66633155764266],[-4.460712421406011,36.6663445786444],[-4.460722724901222,36.66635053409682],[-4.460734422279805,36.66633751309508]]]}},{'type':'Feature','properties':{'area':'G1','block':'0,5'},'geometry':{'type':'Polygon','coordinates':[[[-4.460684298687127,36.66628875937882],[-4.460673995191916,36.6662828039264],[-4.460662297813333,36.66629582492814],[-4.460672601308544,36.666301780380564],[-4.460684298687127,36.66628875937882]]]}}]}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Capítulo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Subcategoría</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Consumo_diario_kWh</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Perfil_24h</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Residencial</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Vivienda Estándar</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Uso General</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>[0.024, 0.016, 0.016, 0.016, 0.016, 0.024, 0.032, 0.145, 0.04, 0.032, 0.024, 0.024, 0.032, 0.04, 0.032, 0.024, 0.032, 0.047, 0.063, 0.08, 0.095, 0.071, 0.047, 0.032]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Residencial</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Vivienda Unifamiliar</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Aire Acondicionado</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>[0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.02, 0.05, 0.08, 0.12, 0.15, 0.15, 0.12, 0.1, 0.08, 0.06, 0.04, 0.02, 0.01, 0.0, 0.0, 0.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Residencial</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Vivienda Unifamiliar</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Calefacción (B. Calor)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>[0.05, 0.06, 0.07, 0.07, 0.07, 0.08, 0.1, 0.12, 0.08, 0.05, 0.03, 0.02, 0.02, 0.02, 0.02, 0.02, 0.02, 0.03, 0.04, 0.05, 0.06, 0.06, 0.04, 0.04]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Residencial</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Vivienda Unifamiliar</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Cargador Coche Eléctrico</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>[0.12, 0.12, 0.12, 0.12, 0.12, 0.12, 0.12, 0.12, 0.04, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.04]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Residencial</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bloque Pisos</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Servicios Comunes</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>[0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Terciario</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Oficina Moderna</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Iluminación LED</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>[0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.05, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.05, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Terciario</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Oficina Moderna</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Climatización</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>[0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.05, 0.1, 0.12, 0.12, 0.12, 0.12, 0.05, 0.12, 0.12, 0.06, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Terciario</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Comercio</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Rótulos Luminosos</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>[0.1, 0.1, 0.1, 0.1, 0.1, 0.05, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.05, 0.1, 0.1, 0.1, 0.1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Nave Producción</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Maquinaria Pesada</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>350</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>[0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.05, 0.15, 0.15, 0.15, 0.15, 0.15, 0.05, 0.15, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Nave Producción</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Aire Comprimido</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>40</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>[0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Almacén Logístico</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Carga Carretillas</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>60</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>[0.1, 0.1, 0.1, 0.1, 0.1, 0.1, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.1, 0.1, 0.1, 0.1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Agrario</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Explotación Agrícola</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Bombeo Riego</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>150</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>[0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.1, 0.15, 0.15, 0.15, 0.15, 0.15, 0.15, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Agrario</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Granja Ganadera</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ventilación Forzada</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>25</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>[0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416, 0.0416]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Agrario</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Granja Ganadera</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Ordeño Automático</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>[0.0, 0.0, 0.0, 0.0, 0.0, 0.2, 0.2, 0.1, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.0, 0.2, 0.2, 0.1, 0.0, 0.0, 0.0, 0.0]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Capítulo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Fijo (€)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>€/Wdc</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>MO (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>Coste Directo</t>
         </is>
       </c>
@@ -718,12 +1532,7 @@
       <c r="E2" t="n">
         <v>0.22</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
+      <c r="F2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -749,12 +1558,7 @@
       <c r="E3" t="n">
         <v>0.12</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
+      <c r="F3" t="n">
         <v>5</v>
       </c>
     </row>
@@ -780,12 +1584,7 @@
       <c r="E4" t="n">
         <v>0.15</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>€/kWh</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
+      <c r="F4" t="n">
         <v>5</v>
       </c>
     </row>
@@ -811,12 +1610,7 @@
       <c r="E5" t="n">
         <v>0.19</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
+      <c r="F5" t="n">
         <v>40</v>
       </c>
     </row>
@@ -842,12 +1636,7 @@
       <c r="E6" t="n">
         <v>0.02</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
+      <c r="F6" t="n">
         <v>10</v>
       </c>
     </row>
@@ -873,12 +1662,7 @@
       <c r="E7" t="n">
         <v>0.005</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
+      <c r="F7" t="n">
         <v>80</v>
       </c>
     </row>
@@ -904,12 +1688,7 @@
       <c r="E8" t="n">
         <v>0.02</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
+      <c r="F8" t="n">
         <v>100</v>
       </c>
     </row>
@@ -935,12 +1714,7 @@
       <c r="E9" t="n">
         <v>0.01</v>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
+      <c r="F9" t="n">
         <v>90</v>
       </c>
     </row>
@@ -966,12 +1740,7 @@
       <c r="E10" t="n">
         <v>0.18</v>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
+      <c r="F10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -997,13 +1766,1058 @@
       <c r="E11" t="n">
         <v>0.04</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>@</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Capítulo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Año_inicio</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Año_fin</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Fijo (€/año)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Unidad_variable</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Operación FV</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Energía fotovoltaica</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PV_Fijo_Anual</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>€/año</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Operación FV</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Energía fotovoltaica</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PV_Fijo_por_Capacidad</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F3" t="n">
+        <v>19</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>€/Wdc</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Operación FV</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Energía fotovoltaica</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PV_Variable_Generacion</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>€/kWh</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Batería</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Almacenamiento</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Bateria_Fijo_Anual</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>15</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>€/año</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Batería</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Almacenamiento</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bateria_Fijo_por_Capacidad</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F6" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>€/kWh_instalada</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Batería</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Almacenamiento</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Bateria_Variable_Descarga</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>15</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>€/kWh_descargado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Batería</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Reemplazo de activos</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bateria_Coste_Reemplazo</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" t="n">
+        <v>252</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>€/kWh_instalada</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Uso de suelo</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Arrendamiento_Anual_Terreno</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>€/año</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>@Otros</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>@Otros</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>@Otros</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>25</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>@€</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Capítulo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Año_inicio</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Año_fin</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Ingreso_fijo (€/año)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Ingreso_variable</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Unidad_variable</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ingresos de explotación</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Autoconsumo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Ahorro autoconsumo</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>€/kWh autoconsumido</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ingresos de explotación</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Excedentes</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Venta excedentes</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>€/kWh exportado</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ingresos de explotación</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Excedentes</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Compensación simplificada</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>€/kWh compensado</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ingresos regulados</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Certificados</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CAE</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>€/kWh generado</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ingresos regulados</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Certificados</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Garantías de origen</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>€/kWh generado</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Subvenciones</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bonificaciones fiscales</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Bonificación IBI</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>€/año</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Subvenciones</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Deducciones fiscales</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Deducción IRPF</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>200</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>€/año</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Subvenciones</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Inversión</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Next Generation</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>% CAPEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Subvenciones</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Locales/autonómicas</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ICIO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>100</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>€/año</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>@Otros</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>@Otros</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>25</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
       <c r="G11" t="n">
         <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>@€</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Capítulo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Categoría</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Parámetro</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Análisis Financiero</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Duración de la actuación</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2033</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>años</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Análisis Financiero</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Impuestos (IVA)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>21</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Análisis Financiero</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mercado</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tasa de inflación</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>%/año</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Análisis Financiero</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mercado</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Precio de la energía</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>€/kWh</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Análisis Financiero</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mercado</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Tasa de descuento (VAN)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Análisis Financiero</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Financiación</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Porcentaje financiado</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>27</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Análisis Financiero</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Financiación</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Años de financiación</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>años</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Análisis Financiero</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Financiación</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Tipo de interés anual</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Análisis Financiero</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Operación</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Tasa seguro anual</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>% de instalación</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>